<commit_message>
Update project: include latest diagnostic graphs and Q-Table reports
</commit_message>
<xml_diff>
--- a/output/v1_teori/Laporan_Q_Table_Lengkap.xlsx
+++ b/output/v1_teori/Laporan_Q_Table_Lengkap.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -417,74 +429,74 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>STATE ID</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>KONDISI LINGKUNGAN</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>0: Idle</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>1: pH Up (S)</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>2: pH Up (L)</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>3: pH Down (S)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>4: pH Down (L)</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>5: Nutrisi (S)</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>6: Nutrisi (L)</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>7: Air Baku (S)</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>8: Air Baku (L)</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>1: pH Up(S)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>2: pH Up(L)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>3: pH Down(S)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>4: pH Down(L)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>5: Nutrisi(S)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>6: Nutrisi(L)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>7: Air Baku(S)</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>8: Air Baku(L)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>KEPUTUSAN AGEN</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>MAX Q-VALUE</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="1" t="n">
         <v>1</v>
       </c>
       <c r="B2" t="inlineStr">
@@ -521,7 +533,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2: pH Up (L)</t>
+          <t>2: pH Up(L)</t>
         </is>
       </c>
       <c r="M2" t="n">
@@ -529,7 +541,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="1" t="n">
         <v>2</v>
       </c>
       <c r="B3" t="inlineStr">
@@ -566,7 +578,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2: pH Up (L)</t>
+          <t>2: pH Up(L)</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -574,7 +586,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="1" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="inlineStr">
@@ -611,7 +623,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2: pH Up (L)</t>
+          <t>2: pH Up(L)</t>
         </is>
       </c>
       <c r="M4" t="n">
@@ -619,7 +631,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="1" t="n">
         <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
@@ -656,7 +668,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2: pH Up (L)</t>
+          <t>2: pH Up(L)</t>
         </is>
       </c>
       <c r="M5" t="n">
@@ -664,7 +676,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
@@ -701,7 +713,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>8: Air Baku (L)</t>
+          <t>8: Air Baku(L)</t>
         </is>
       </c>
       <c r="M6" t="n">
@@ -709,7 +721,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="1" t="n">
         <v>6</v>
       </c>
       <c r="B7" t="inlineStr">
@@ -746,7 +758,7 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>6: Nutrisi (L)</t>
+          <t>6: Nutrisi(L)</t>
         </is>
       </c>
       <c r="M7" t="n">
@@ -754,7 +766,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="1" t="n">
         <v>7</v>
       </c>
       <c r="B8" t="inlineStr">
@@ -791,7 +803,7 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>6: Nutrisi (L)</t>
+          <t>6: Nutrisi(L)</t>
         </is>
       </c>
       <c r="M8" t="n">
@@ -799,7 +811,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="1" t="n">
         <v>8</v>
       </c>
       <c r="B9" t="inlineStr">
@@ -836,7 +848,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>2: pH Up (L)</t>
+          <t>2: pH Up(L)</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -844,7 +856,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="1" t="n">
         <v>9</v>
       </c>
       <c r="B10" t="inlineStr">
@@ -881,7 +893,7 @@
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>1: pH Up (S)</t>
+          <t>1: pH Up(S)</t>
         </is>
       </c>
       <c r="M10" t="n">
@@ -889,7 +901,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="1" t="n">
         <v>10</v>
       </c>
       <c r="B11" t="inlineStr">
@@ -926,7 +938,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>7: Air Baku (S)</t>
+          <t>7: Air Baku(S)</t>
         </is>
       </c>
       <c r="M11" t="n">
@@ -934,7 +946,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="1" t="n">
         <v>11</v>
       </c>
       <c r="B12" t="inlineStr">
@@ -971,7 +983,7 @@
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>6: Nutrisi (L)</t>
+          <t>6: Nutrisi(L)</t>
         </is>
       </c>
       <c r="M12" t="n">
@@ -979,7 +991,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="1" t="n">
         <v>12</v>
       </c>
       <c r="B13" t="inlineStr">
@@ -1016,7 +1028,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>5: Nutrisi (S)</t>
+          <t>5: Nutrisi(S)</t>
         </is>
       </c>
       <c r="M13" t="n">
@@ -1024,7 +1036,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="1" t="n">
         <v>13</v>
       </c>
       <c r="B14" t="inlineStr">
@@ -1069,7 +1081,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="1" t="n">
         <v>14</v>
       </c>
       <c r="B15" t="inlineStr">
@@ -1106,7 +1118,7 @@
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>7: Air Baku (S)</t>
+          <t>7: Air Baku(S)</t>
         </is>
       </c>
       <c r="M15" t="n">
@@ -1114,7 +1126,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="1" t="n">
         <v>15</v>
       </c>
       <c r="B16" t="inlineStr">
@@ -1151,7 +1163,7 @@
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>8: Air Baku (L)</t>
+          <t>8: Air Baku(L)</t>
         </is>
       </c>
       <c r="M16" t="n">
@@ -1159,7 +1171,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="1" t="n">
         <v>16</v>
       </c>
       <c r="B17" t="inlineStr">
@@ -1196,7 +1208,7 @@
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>6: Nutrisi (L)</t>
+          <t>6: Nutrisi(L)</t>
         </is>
       </c>
       <c r="M17" t="n">
@@ -1204,7 +1216,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="1" t="n">
         <v>17</v>
       </c>
       <c r="B18" t="inlineStr">
@@ -1241,7 +1253,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M18" t="n">
@@ -1249,7 +1261,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="1" t="n">
         <v>18</v>
       </c>
       <c r="B19" t="inlineStr">
@@ -1286,7 +1298,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M19" t="n">
@@ -1294,7 +1306,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="1" t="n">
         <v>19</v>
       </c>
       <c r="B20" t="inlineStr">
@@ -1331,7 +1343,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M20" t="n">
@@ -1339,7 +1351,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="1" t="n">
         <v>20</v>
       </c>
       <c r="B21" t="inlineStr">
@@ -1376,7 +1388,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>8: Air Baku (L)</t>
+          <t>8: Air Baku(L)</t>
         </is>
       </c>
       <c r="M21" t="n">
@@ -1384,7 +1396,7 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="1" t="n">
         <v>21</v>
       </c>
       <c r="B22" t="inlineStr">
@@ -1421,7 +1433,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>6: Nutrisi (L)</t>
+          <t>6: Nutrisi(L)</t>
         </is>
       </c>
       <c r="M22" t="n">
@@ -1429,7 +1441,7 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="1" t="n">
         <v>22</v>
       </c>
       <c r="B23" t="inlineStr">
@@ -1466,7 +1478,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -1474,7 +1486,7 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="n">
+      <c r="A24" s="1" t="n">
         <v>23</v>
       </c>
       <c r="B24" t="inlineStr">
@@ -1511,7 +1523,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M24" t="n">
@@ -1519,7 +1531,7 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="n">
+      <c r="A25" s="1" t="n">
         <v>24</v>
       </c>
       <c r="B25" t="inlineStr">
@@ -1556,7 +1568,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M25" t="n">
@@ -1564,7 +1576,7 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="n">
+      <c r="A26" s="1" t="n">
         <v>25</v>
       </c>
       <c r="B26" t="inlineStr">
@@ -1601,7 +1613,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>4: pH Down (L)</t>
+          <t>4: pH Down(L)</t>
         </is>
       </c>
       <c r="M26" t="n">

</xml_diff>